<commit_message>
Add required RFC field for users and reports
</commit_message>
<xml_diff>
--- a/outputs/godaddy_prueba/admin/assets/layout_carga_usuarios.xlsx
+++ b/outputs/godaddy_prueba/admin/assets/layout_carga_usuarios.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Promotores'!$A$1:$F$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Instrucciones'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Promotores'!$A$1:$G$503</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Instrucciones'!$A$1:$C$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -184,15 +184,20 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Telefono del promotor. Obligatorio.</t>
+        <t>RFC del promotor. Obligatorio para historico y busqueda.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
+        <t>Telefono del promotor. Obligatorio.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
         <t>Opcional. Puede ser nombre, email o numero de empleado del supervisor. Los supervisores pueden ver a todos los promotores.</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Opcional si se define contrasena default en el panel. Minimo recomendado: 8 caracteres.</t>
       </text>
@@ -490,15 +495,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F503"/>
+  <dimension ref="A1:G503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,15 +525,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>telefono</t>
+          <t>rfc</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>telefono</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>supervisor</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>contrasena</t>
         </is>
@@ -551,11 +562,16 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>PRO101010AAA</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>5512340001</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Cambiar123!</t>
         </is>
@@ -579,15 +595,20 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>5512340002</t>
+          <t>PRO102010AAA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>5512340002</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Supervisor 1</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Cambiar123!</t>
         </is>
@@ -611,15 +632,20 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>5512340003</t>
+          <t>PRO103010AAA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>5512340003</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>supervisor1@sealy.com</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Cambiar123!</t>
         </is>
@@ -632,6 +658,7 @@
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -640,6 +667,7 @@
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -648,6 +676,7 @@
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -656,6 +685,7 @@
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -664,6 +694,7 @@
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -672,6 +703,7 @@
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -680,6 +712,7 @@
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -688,6 +721,7 @@
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -696,6 +730,7 @@
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -704,6 +739,7 @@
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -712,6 +748,7 @@
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -720,6 +757,7 @@
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -728,6 +766,7 @@
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -736,6 +775,7 @@
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -744,6 +784,7 @@
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -752,6 +793,7 @@
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -760,6 +802,7 @@
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -768,6 +811,7 @@
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -776,6 +820,7 @@
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -784,6 +829,7 @@
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -792,6 +838,7 @@
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -800,6 +847,7 @@
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -808,6 +856,7 @@
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -816,6 +865,7 @@
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -824,6 +874,7 @@
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -832,6 +883,7 @@
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -840,6 +892,7 @@
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -848,6 +901,7 @@
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -856,6 +910,7 @@
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -864,6 +919,7 @@
       <c r="D34" s="2" t="n"/>
       <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -872,6 +928,7 @@
       <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -880,6 +937,7 @@
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -888,6 +946,7 @@
       <c r="D37" s="2" t="n"/>
       <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -896,6 +955,7 @@
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -904,6 +964,7 @@
       <c r="D39" s="2" t="n"/>
       <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -912,6 +973,7 @@
       <c r="D40" s="2" t="n"/>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -920,6 +982,7 @@
       <c r="D41" s="2" t="n"/>
       <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -928,6 +991,7 @@
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -936,6 +1000,7 @@
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -944,6 +1009,7 @@
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -952,6 +1018,7 @@
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -960,6 +1027,7 @@
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -968,6 +1036,7 @@
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -976,6 +1045,7 @@
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -984,6 +1054,7 @@
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -992,6 +1063,7 @@
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1000,6 +1072,7 @@
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1008,6 +1081,7 @@
       <c r="D52" s="2" t="n"/>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1016,6 +1090,7 @@
       <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1024,6 +1099,7 @@
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1032,6 +1108,7 @@
       <c r="D55" s="2" t="n"/>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1040,6 +1117,7 @@
       <c r="D56" s="2" t="n"/>
       <c r="E56" s="2" t="n"/>
       <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1048,6 +1126,7 @@
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1056,6 +1135,7 @@
       <c r="D58" s="2" t="n"/>
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1064,6 +1144,7 @@
       <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1072,6 +1153,7 @@
       <c r="D60" s="2" t="n"/>
       <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1080,6 +1162,7 @@
       <c r="D61" s="2" t="n"/>
       <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1088,6 +1171,7 @@
       <c r="D62" s="2" t="n"/>
       <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1096,6 +1180,7 @@
       <c r="D63" s="2" t="n"/>
       <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1104,6 +1189,7 @@
       <c r="D64" s="2" t="n"/>
       <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1112,6 +1198,7 @@
       <c r="D65" s="2" t="n"/>
       <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1120,6 +1207,7 @@
       <c r="D66" s="2" t="n"/>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1128,6 +1216,7 @@
       <c r="D67" s="2" t="n"/>
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1136,6 +1225,7 @@
       <c r="D68" s="2" t="n"/>
       <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1144,6 +1234,7 @@
       <c r="D69" s="2" t="n"/>
       <c r="E69" s="2" t="n"/>
       <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1152,6 +1243,7 @@
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1160,6 +1252,7 @@
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1168,6 +1261,7 @@
       <c r="D72" s="2" t="n"/>
       <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1176,6 +1270,7 @@
       <c r="D73" s="2" t="n"/>
       <c r="E73" s="2" t="n"/>
       <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1184,6 +1279,7 @@
       <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="n"/>
       <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1192,6 +1288,7 @@
       <c r="D75" s="2" t="n"/>
       <c r="E75" s="2" t="n"/>
       <c r="F75" s="2" t="n"/>
+      <c r="G75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1200,6 +1297,7 @@
       <c r="D76" s="2" t="n"/>
       <c r="E76" s="2" t="n"/>
       <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1208,6 +1306,7 @@
       <c r="D77" s="2" t="n"/>
       <c r="E77" s="2" t="n"/>
       <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1216,6 +1315,7 @@
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
       <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1224,6 +1324,7 @@
       <c r="D79" s="2" t="n"/>
       <c r="E79" s="2" t="n"/>
       <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1232,6 +1333,7 @@
       <c r="D80" s="2" t="n"/>
       <c r="E80" s="2" t="n"/>
       <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1240,6 +1342,7 @@
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1248,6 +1351,7 @@
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="n"/>
       <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1256,6 +1360,7 @@
       <c r="D83" s="2" t="n"/>
       <c r="E83" s="2" t="n"/>
       <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1264,6 +1369,7 @@
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="2" t="n"/>
       <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1272,6 +1378,7 @@
       <c r="D85" s="2" t="n"/>
       <c r="E85" s="2" t="n"/>
       <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1280,6 +1387,7 @@
       <c r="D86" s="2" t="n"/>
       <c r="E86" s="2" t="n"/>
       <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1288,6 +1396,7 @@
       <c r="D87" s="2" t="n"/>
       <c r="E87" s="2" t="n"/>
       <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1296,6 +1405,7 @@
       <c r="D88" s="2" t="n"/>
       <c r="E88" s="2" t="n"/>
       <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -1304,6 +1414,7 @@
       <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="n"/>
+      <c r="G89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -1312,6 +1423,7 @@
       <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -1320,6 +1432,7 @@
       <c r="D91" s="2" t="n"/>
       <c r="E91" s="2" t="n"/>
       <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -1328,6 +1441,7 @@
       <c r="D92" s="2" t="n"/>
       <c r="E92" s="2" t="n"/>
       <c r="F92" s="2" t="n"/>
+      <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -1336,6 +1450,7 @@
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="2" t="n"/>
       <c r="F93" s="2" t="n"/>
+      <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -1344,6 +1459,7 @@
       <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
       <c r="F94" s="2" t="n"/>
+      <c r="G94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -1352,6 +1468,7 @@
       <c r="D95" s="2" t="n"/>
       <c r="E95" s="2" t="n"/>
       <c r="F95" s="2" t="n"/>
+      <c r="G95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -1360,6 +1477,7 @@
       <c r="D96" s="2" t="n"/>
       <c r="E96" s="2" t="n"/>
       <c r="F96" s="2" t="n"/>
+      <c r="G96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -1368,6 +1486,7 @@
       <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
       <c r="F97" s="2" t="n"/>
+      <c r="G97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -1376,6 +1495,7 @@
       <c r="D98" s="2" t="n"/>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="n"/>
+      <c r="G98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -1384,6 +1504,7 @@
       <c r="D99" s="2" t="n"/>
       <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
+      <c r="G99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -1392,6 +1513,7 @@
       <c r="D100" s="2" t="n"/>
       <c r="E100" s="2" t="n"/>
       <c r="F100" s="2" t="n"/>
+      <c r="G100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -1400,6 +1522,7 @@
       <c r="D101" s="2" t="n"/>
       <c r="E101" s="2" t="n"/>
       <c r="F101" s="2" t="n"/>
+      <c r="G101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -1408,6 +1531,7 @@
       <c r="D102" s="2" t="n"/>
       <c r="E102" s="2" t="n"/>
       <c r="F102" s="2" t="n"/>
+      <c r="G102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -1416,6 +1540,7 @@
       <c r="D103" s="2" t="n"/>
       <c r="E103" s="2" t="n"/>
       <c r="F103" s="2" t="n"/>
+      <c r="G103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -1424,6 +1549,7 @@
       <c r="D104" s="2" t="n"/>
       <c r="E104" s="2" t="n"/>
       <c r="F104" s="2" t="n"/>
+      <c r="G104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -1432,6 +1558,7 @@
       <c r="D105" s="2" t="n"/>
       <c r="E105" s="2" t="n"/>
       <c r="F105" s="2" t="n"/>
+      <c r="G105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -1440,6 +1567,7 @@
       <c r="D106" s="2" t="n"/>
       <c r="E106" s="2" t="n"/>
       <c r="F106" s="2" t="n"/>
+      <c r="G106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -1448,6 +1576,7 @@
       <c r="D107" s="2" t="n"/>
       <c r="E107" s="2" t="n"/>
       <c r="F107" s="2" t="n"/>
+      <c r="G107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -1456,6 +1585,7 @@
       <c r="D108" s="2" t="n"/>
       <c r="E108" s="2" t="n"/>
       <c r="F108" s="2" t="n"/>
+      <c r="G108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -1464,6 +1594,7 @@
       <c r="D109" s="2" t="n"/>
       <c r="E109" s="2" t="n"/>
       <c r="F109" s="2" t="n"/>
+      <c r="G109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -1472,6 +1603,7 @@
       <c r="D110" s="2" t="n"/>
       <c r="E110" s="2" t="n"/>
       <c r="F110" s="2" t="n"/>
+      <c r="G110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -1480,6 +1612,7 @@
       <c r="D111" s="2" t="n"/>
       <c r="E111" s="2" t="n"/>
       <c r="F111" s="2" t="n"/>
+      <c r="G111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -1488,6 +1621,7 @@
       <c r="D112" s="2" t="n"/>
       <c r="E112" s="2" t="n"/>
       <c r="F112" s="2" t="n"/>
+      <c r="G112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -1496,6 +1630,7 @@
       <c r="D113" s="2" t="n"/>
       <c r="E113" s="2" t="n"/>
       <c r="F113" s="2" t="n"/>
+      <c r="G113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -1504,6 +1639,7 @@
       <c r="D114" s="2" t="n"/>
       <c r="E114" s="2" t="n"/>
       <c r="F114" s="2" t="n"/>
+      <c r="G114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -1512,6 +1648,7 @@
       <c r="D115" s="2" t="n"/>
       <c r="E115" s="2" t="n"/>
       <c r="F115" s="2" t="n"/>
+      <c r="G115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -1520,6 +1657,7 @@
       <c r="D116" s="2" t="n"/>
       <c r="E116" s="2" t="n"/>
       <c r="F116" s="2" t="n"/>
+      <c r="G116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -1528,6 +1666,7 @@
       <c r="D117" s="2" t="n"/>
       <c r="E117" s="2" t="n"/>
       <c r="F117" s="2" t="n"/>
+      <c r="G117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -1536,6 +1675,7 @@
       <c r="D118" s="2" t="n"/>
       <c r="E118" s="2" t="n"/>
       <c r="F118" s="2" t="n"/>
+      <c r="G118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -1544,6 +1684,7 @@
       <c r="D119" s="2" t="n"/>
       <c r="E119" s="2" t="n"/>
       <c r="F119" s="2" t="n"/>
+      <c r="G119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -1552,6 +1693,7 @@
       <c r="D120" s="2" t="n"/>
       <c r="E120" s="2" t="n"/>
       <c r="F120" s="2" t="n"/>
+      <c r="G120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -1560,6 +1702,7 @@
       <c r="D121" s="2" t="n"/>
       <c r="E121" s="2" t="n"/>
       <c r="F121" s="2" t="n"/>
+      <c r="G121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -1568,6 +1711,7 @@
       <c r="D122" s="2" t="n"/>
       <c r="E122" s="2" t="n"/>
       <c r="F122" s="2" t="n"/>
+      <c r="G122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -1576,6 +1720,7 @@
       <c r="D123" s="2" t="n"/>
       <c r="E123" s="2" t="n"/>
       <c r="F123" s="2" t="n"/>
+      <c r="G123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -1584,6 +1729,7 @@
       <c r="D124" s="2" t="n"/>
       <c r="E124" s="2" t="n"/>
       <c r="F124" s="2" t="n"/>
+      <c r="G124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -1592,6 +1738,7 @@
       <c r="D125" s="2" t="n"/>
       <c r="E125" s="2" t="n"/>
       <c r="F125" s="2" t="n"/>
+      <c r="G125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -1600,6 +1747,7 @@
       <c r="D126" s="2" t="n"/>
       <c r="E126" s="2" t="n"/>
       <c r="F126" s="2" t="n"/>
+      <c r="G126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -1608,6 +1756,7 @@
       <c r="D127" s="2" t="n"/>
       <c r="E127" s="2" t="n"/>
       <c r="F127" s="2" t="n"/>
+      <c r="G127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -1616,6 +1765,7 @@
       <c r="D128" s="2" t="n"/>
       <c r="E128" s="2" t="n"/>
       <c r="F128" s="2" t="n"/>
+      <c r="G128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -1624,6 +1774,7 @@
       <c r="D129" s="2" t="n"/>
       <c r="E129" s="2" t="n"/>
       <c r="F129" s="2" t="n"/>
+      <c r="G129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -1632,6 +1783,7 @@
       <c r="D130" s="2" t="n"/>
       <c r="E130" s="2" t="n"/>
       <c r="F130" s="2" t="n"/>
+      <c r="G130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -1640,6 +1792,7 @@
       <c r="D131" s="2" t="n"/>
       <c r="E131" s="2" t="n"/>
       <c r="F131" s="2" t="n"/>
+      <c r="G131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -1648,6 +1801,7 @@
       <c r="D132" s="2" t="n"/>
       <c r="E132" s="2" t="n"/>
       <c r="F132" s="2" t="n"/>
+      <c r="G132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -1656,6 +1810,7 @@
       <c r="D133" s="2" t="n"/>
       <c r="E133" s="2" t="n"/>
       <c r="F133" s="2" t="n"/>
+      <c r="G133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -1664,6 +1819,7 @@
       <c r="D134" s="2" t="n"/>
       <c r="E134" s="2" t="n"/>
       <c r="F134" s="2" t="n"/>
+      <c r="G134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -1672,6 +1828,7 @@
       <c r="D135" s="2" t="n"/>
       <c r="E135" s="2" t="n"/>
       <c r="F135" s="2" t="n"/>
+      <c r="G135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -1680,6 +1837,7 @@
       <c r="D136" s="2" t="n"/>
       <c r="E136" s="2" t="n"/>
       <c r="F136" s="2" t="n"/>
+      <c r="G136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -1688,6 +1846,7 @@
       <c r="D137" s="2" t="n"/>
       <c r="E137" s="2" t="n"/>
       <c r="F137" s="2" t="n"/>
+      <c r="G137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -1696,6 +1855,7 @@
       <c r="D138" s="2" t="n"/>
       <c r="E138" s="2" t="n"/>
       <c r="F138" s="2" t="n"/>
+      <c r="G138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -1704,6 +1864,7 @@
       <c r="D139" s="2" t="n"/>
       <c r="E139" s="2" t="n"/>
       <c r="F139" s="2" t="n"/>
+      <c r="G139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -1712,6 +1873,7 @@
       <c r="D140" s="2" t="n"/>
       <c r="E140" s="2" t="n"/>
       <c r="F140" s="2" t="n"/>
+      <c r="G140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -1720,6 +1882,7 @@
       <c r="D141" s="2" t="n"/>
       <c r="E141" s="2" t="n"/>
       <c r="F141" s="2" t="n"/>
+      <c r="G141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -1728,6 +1891,7 @@
       <c r="D142" s="2" t="n"/>
       <c r="E142" s="2" t="n"/>
       <c r="F142" s="2" t="n"/>
+      <c r="G142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -1736,6 +1900,7 @@
       <c r="D143" s="2" t="n"/>
       <c r="E143" s="2" t="n"/>
       <c r="F143" s="2" t="n"/>
+      <c r="G143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -1744,6 +1909,7 @@
       <c r="D144" s="2" t="n"/>
       <c r="E144" s="2" t="n"/>
       <c r="F144" s="2" t="n"/>
+      <c r="G144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -1752,6 +1918,7 @@
       <c r="D145" s="2" t="n"/>
       <c r="E145" s="2" t="n"/>
       <c r="F145" s="2" t="n"/>
+      <c r="G145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -1760,6 +1927,7 @@
       <c r="D146" s="2" t="n"/>
       <c r="E146" s="2" t="n"/>
       <c r="F146" s="2" t="n"/>
+      <c r="G146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -1768,6 +1936,7 @@
       <c r="D147" s="2" t="n"/>
       <c r="E147" s="2" t="n"/>
       <c r="F147" s="2" t="n"/>
+      <c r="G147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -1776,6 +1945,7 @@
       <c r="D148" s="2" t="n"/>
       <c r="E148" s="2" t="n"/>
       <c r="F148" s="2" t="n"/>
+      <c r="G148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -1784,6 +1954,7 @@
       <c r="D149" s="2" t="n"/>
       <c r="E149" s="2" t="n"/>
       <c r="F149" s="2" t="n"/>
+      <c r="G149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -1792,6 +1963,7 @@
       <c r="D150" s="2" t="n"/>
       <c r="E150" s="2" t="n"/>
       <c r="F150" s="2" t="n"/>
+      <c r="G150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -1800,6 +1972,7 @@
       <c r="D151" s="2" t="n"/>
       <c r="E151" s="2" t="n"/>
       <c r="F151" s="2" t="n"/>
+      <c r="G151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -1808,6 +1981,7 @@
       <c r="D152" s="2" t="n"/>
       <c r="E152" s="2" t="n"/>
       <c r="F152" s="2" t="n"/>
+      <c r="G152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -1816,6 +1990,7 @@
       <c r="D153" s="2" t="n"/>
       <c r="E153" s="2" t="n"/>
       <c r="F153" s="2" t="n"/>
+      <c r="G153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -1824,6 +1999,7 @@
       <c r="D154" s="2" t="n"/>
       <c r="E154" s="2" t="n"/>
       <c r="F154" s="2" t="n"/>
+      <c r="G154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -1832,6 +2008,7 @@
       <c r="D155" s="2" t="n"/>
       <c r="E155" s="2" t="n"/>
       <c r="F155" s="2" t="n"/>
+      <c r="G155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -1840,6 +2017,7 @@
       <c r="D156" s="2" t="n"/>
       <c r="E156" s="2" t="n"/>
       <c r="F156" s="2" t="n"/>
+      <c r="G156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -1848,6 +2026,7 @@
       <c r="D157" s="2" t="n"/>
       <c r="E157" s="2" t="n"/>
       <c r="F157" s="2" t="n"/>
+      <c r="G157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -1856,6 +2035,7 @@
       <c r="D158" s="2" t="n"/>
       <c r="E158" s="2" t="n"/>
       <c r="F158" s="2" t="n"/>
+      <c r="G158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -1864,6 +2044,7 @@
       <c r="D159" s="2" t="n"/>
       <c r="E159" s="2" t="n"/>
       <c r="F159" s="2" t="n"/>
+      <c r="G159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -1872,6 +2053,7 @@
       <c r="D160" s="2" t="n"/>
       <c r="E160" s="2" t="n"/>
       <c r="F160" s="2" t="n"/>
+      <c r="G160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -1880,6 +2062,7 @@
       <c r="D161" s="2" t="n"/>
       <c r="E161" s="2" t="n"/>
       <c r="F161" s="2" t="n"/>
+      <c r="G161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -1888,6 +2071,7 @@
       <c r="D162" s="2" t="n"/>
       <c r="E162" s="2" t="n"/>
       <c r="F162" s="2" t="n"/>
+      <c r="G162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -1896,6 +2080,7 @@
       <c r="D163" s="2" t="n"/>
       <c r="E163" s="2" t="n"/>
       <c r="F163" s="2" t="n"/>
+      <c r="G163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -1904,6 +2089,7 @@
       <c r="D164" s="2" t="n"/>
       <c r="E164" s="2" t="n"/>
       <c r="F164" s="2" t="n"/>
+      <c r="G164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -1912,6 +2098,7 @@
       <c r="D165" s="2" t="n"/>
       <c r="E165" s="2" t="n"/>
       <c r="F165" s="2" t="n"/>
+      <c r="G165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -1920,6 +2107,7 @@
       <c r="D166" s="2" t="n"/>
       <c r="E166" s="2" t="n"/>
       <c r="F166" s="2" t="n"/>
+      <c r="G166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -1928,6 +2116,7 @@
       <c r="D167" s="2" t="n"/>
       <c r="E167" s="2" t="n"/>
       <c r="F167" s="2" t="n"/>
+      <c r="G167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -1936,6 +2125,7 @@
       <c r="D168" s="2" t="n"/>
       <c r="E168" s="2" t="n"/>
       <c r="F168" s="2" t="n"/>
+      <c r="G168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -1944,6 +2134,7 @@
       <c r="D169" s="2" t="n"/>
       <c r="E169" s="2" t="n"/>
       <c r="F169" s="2" t="n"/>
+      <c r="G169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -1952,6 +2143,7 @@
       <c r="D170" s="2" t="n"/>
       <c r="E170" s="2" t="n"/>
       <c r="F170" s="2" t="n"/>
+      <c r="G170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -1960,6 +2152,7 @@
       <c r="D171" s="2" t="n"/>
       <c r="E171" s="2" t="n"/>
       <c r="F171" s="2" t="n"/>
+      <c r="G171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -1968,6 +2161,7 @@
       <c r="D172" s="2" t="n"/>
       <c r="E172" s="2" t="n"/>
       <c r="F172" s="2" t="n"/>
+      <c r="G172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -1976,6 +2170,7 @@
       <c r="D173" s="2" t="n"/>
       <c r="E173" s="2" t="n"/>
       <c r="F173" s="2" t="n"/>
+      <c r="G173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -1984,6 +2179,7 @@
       <c r="D174" s="2" t="n"/>
       <c r="E174" s="2" t="n"/>
       <c r="F174" s="2" t="n"/>
+      <c r="G174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -1992,6 +2188,7 @@
       <c r="D175" s="2" t="n"/>
       <c r="E175" s="2" t="n"/>
       <c r="F175" s="2" t="n"/>
+      <c r="G175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -2000,6 +2197,7 @@
       <c r="D176" s="2" t="n"/>
       <c r="E176" s="2" t="n"/>
       <c r="F176" s="2" t="n"/>
+      <c r="G176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -2008,6 +2206,7 @@
       <c r="D177" s="2" t="n"/>
       <c r="E177" s="2" t="n"/>
       <c r="F177" s="2" t="n"/>
+      <c r="G177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -2016,6 +2215,7 @@
       <c r="D178" s="2" t="n"/>
       <c r="E178" s="2" t="n"/>
       <c r="F178" s="2" t="n"/>
+      <c r="G178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -2024,6 +2224,7 @@
       <c r="D179" s="2" t="n"/>
       <c r="E179" s="2" t="n"/>
       <c r="F179" s="2" t="n"/>
+      <c r="G179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -2032,6 +2233,7 @@
       <c r="D180" s="2" t="n"/>
       <c r="E180" s="2" t="n"/>
       <c r="F180" s="2" t="n"/>
+      <c r="G180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -2040,6 +2242,7 @@
       <c r="D181" s="2" t="n"/>
       <c r="E181" s="2" t="n"/>
       <c r="F181" s="2" t="n"/>
+      <c r="G181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -2048,6 +2251,7 @@
       <c r="D182" s="2" t="n"/>
       <c r="E182" s="2" t="n"/>
       <c r="F182" s="2" t="n"/>
+      <c r="G182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -2056,6 +2260,7 @@
       <c r="D183" s="2" t="n"/>
       <c r="E183" s="2" t="n"/>
       <c r="F183" s="2" t="n"/>
+      <c r="G183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -2064,6 +2269,7 @@
       <c r="D184" s="2" t="n"/>
       <c r="E184" s="2" t="n"/>
       <c r="F184" s="2" t="n"/>
+      <c r="G184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -2072,6 +2278,7 @@
       <c r="D185" s="2" t="n"/>
       <c r="E185" s="2" t="n"/>
       <c r="F185" s="2" t="n"/>
+      <c r="G185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -2080,6 +2287,7 @@
       <c r="D186" s="2" t="n"/>
       <c r="E186" s="2" t="n"/>
       <c r="F186" s="2" t="n"/>
+      <c r="G186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -2088,6 +2296,7 @@
       <c r="D187" s="2" t="n"/>
       <c r="E187" s="2" t="n"/>
       <c r="F187" s="2" t="n"/>
+      <c r="G187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -2096,6 +2305,7 @@
       <c r="D188" s="2" t="n"/>
       <c r="E188" s="2" t="n"/>
       <c r="F188" s="2" t="n"/>
+      <c r="G188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -2104,6 +2314,7 @@
       <c r="D189" s="2" t="n"/>
       <c r="E189" s="2" t="n"/>
       <c r="F189" s="2" t="n"/>
+      <c r="G189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -2112,6 +2323,7 @@
       <c r="D190" s="2" t="n"/>
       <c r="E190" s="2" t="n"/>
       <c r="F190" s="2" t="n"/>
+      <c r="G190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -2120,6 +2332,7 @@
       <c r="D191" s="2" t="n"/>
       <c r="E191" s="2" t="n"/>
       <c r="F191" s="2" t="n"/>
+      <c r="G191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -2128,6 +2341,7 @@
       <c r="D192" s="2" t="n"/>
       <c r="E192" s="2" t="n"/>
       <c r="F192" s="2" t="n"/>
+      <c r="G192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -2136,6 +2350,7 @@
       <c r="D193" s="2" t="n"/>
       <c r="E193" s="2" t="n"/>
       <c r="F193" s="2" t="n"/>
+      <c r="G193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -2144,6 +2359,7 @@
       <c r="D194" s="2" t="n"/>
       <c r="E194" s="2" t="n"/>
       <c r="F194" s="2" t="n"/>
+      <c r="G194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -2152,6 +2368,7 @@
       <c r="D195" s="2" t="n"/>
       <c r="E195" s="2" t="n"/>
       <c r="F195" s="2" t="n"/>
+      <c r="G195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -2160,6 +2377,7 @@
       <c r="D196" s="2" t="n"/>
       <c r="E196" s="2" t="n"/>
       <c r="F196" s="2" t="n"/>
+      <c r="G196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -2168,6 +2386,7 @@
       <c r="D197" s="2" t="n"/>
       <c r="E197" s="2" t="n"/>
       <c r="F197" s="2" t="n"/>
+      <c r="G197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -2176,6 +2395,7 @@
       <c r="D198" s="2" t="n"/>
       <c r="E198" s="2" t="n"/>
       <c r="F198" s="2" t="n"/>
+      <c r="G198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -2184,6 +2404,7 @@
       <c r="D199" s="2" t="n"/>
       <c r="E199" s="2" t="n"/>
       <c r="F199" s="2" t="n"/>
+      <c r="G199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -2192,6 +2413,7 @@
       <c r="D200" s="2" t="n"/>
       <c r="E200" s="2" t="n"/>
       <c r="F200" s="2" t="n"/>
+      <c r="G200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
@@ -2200,6 +2422,7 @@
       <c r="D201" s="2" t="n"/>
       <c r="E201" s="2" t="n"/>
       <c r="F201" s="2" t="n"/>
+      <c r="G201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n"/>
@@ -2208,6 +2431,7 @@
       <c r="D202" s="2" t="n"/>
       <c r="E202" s="2" t="n"/>
       <c r="F202" s="2" t="n"/>
+      <c r="G202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n"/>
@@ -2216,6 +2440,7 @@
       <c r="D203" s="2" t="n"/>
       <c r="E203" s="2" t="n"/>
       <c r="F203" s="2" t="n"/>
+      <c r="G203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n"/>
@@ -2224,6 +2449,7 @@
       <c r="D204" s="2" t="n"/>
       <c r="E204" s="2" t="n"/>
       <c r="F204" s="2" t="n"/>
+      <c r="G204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n"/>
@@ -2232,6 +2458,7 @@
       <c r="D205" s="2" t="n"/>
       <c r="E205" s="2" t="n"/>
       <c r="F205" s="2" t="n"/>
+      <c r="G205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n"/>
@@ -2240,6 +2467,7 @@
       <c r="D206" s="2" t="n"/>
       <c r="E206" s="2" t="n"/>
       <c r="F206" s="2" t="n"/>
+      <c r="G206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n"/>
@@ -2248,6 +2476,7 @@
       <c r="D207" s="2" t="n"/>
       <c r="E207" s="2" t="n"/>
       <c r="F207" s="2" t="n"/>
+      <c r="G207" s="2" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n"/>
@@ -2256,6 +2485,7 @@
       <c r="D208" s="2" t="n"/>
       <c r="E208" s="2" t="n"/>
       <c r="F208" s="2" t="n"/>
+      <c r="G208" s="2" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n"/>
@@ -2264,6 +2494,7 @@
       <c r="D209" s="2" t="n"/>
       <c r="E209" s="2" t="n"/>
       <c r="F209" s="2" t="n"/>
+      <c r="G209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n"/>
@@ -2272,6 +2503,7 @@
       <c r="D210" s="2" t="n"/>
       <c r="E210" s="2" t="n"/>
       <c r="F210" s="2" t="n"/>
+      <c r="G210" s="2" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n"/>
@@ -2280,6 +2512,7 @@
       <c r="D211" s="2" t="n"/>
       <c r="E211" s="2" t="n"/>
       <c r="F211" s="2" t="n"/>
+      <c r="G211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n"/>
@@ -2288,6 +2521,7 @@
       <c r="D212" s="2" t="n"/>
       <c r="E212" s="2" t="n"/>
       <c r="F212" s="2" t="n"/>
+      <c r="G212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n"/>
@@ -2296,6 +2530,7 @@
       <c r="D213" s="2" t="n"/>
       <c r="E213" s="2" t="n"/>
       <c r="F213" s="2" t="n"/>
+      <c r="G213" s="2" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n"/>
@@ -2304,6 +2539,7 @@
       <c r="D214" s="2" t="n"/>
       <c r="E214" s="2" t="n"/>
       <c r="F214" s="2" t="n"/>
+      <c r="G214" s="2" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n"/>
@@ -2312,6 +2548,7 @@
       <c r="D215" s="2" t="n"/>
       <c r="E215" s="2" t="n"/>
       <c r="F215" s="2" t="n"/>
+      <c r="G215" s="2" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n"/>
@@ -2320,6 +2557,7 @@
       <c r="D216" s="2" t="n"/>
       <c r="E216" s="2" t="n"/>
       <c r="F216" s="2" t="n"/>
+      <c r="G216" s="2" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n"/>
@@ -2328,6 +2566,7 @@
       <c r="D217" s="2" t="n"/>
       <c r="E217" s="2" t="n"/>
       <c r="F217" s="2" t="n"/>
+      <c r="G217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n"/>
@@ -2336,6 +2575,7 @@
       <c r="D218" s="2" t="n"/>
       <c r="E218" s="2" t="n"/>
       <c r="F218" s="2" t="n"/>
+      <c r="G218" s="2" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n"/>
@@ -2344,6 +2584,7 @@
       <c r="D219" s="2" t="n"/>
       <c r="E219" s="2" t="n"/>
       <c r="F219" s="2" t="n"/>
+      <c r="G219" s="2" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n"/>
@@ -2352,6 +2593,7 @@
       <c r="D220" s="2" t="n"/>
       <c r="E220" s="2" t="n"/>
       <c r="F220" s="2" t="n"/>
+      <c r="G220" s="2" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n"/>
@@ -2360,6 +2602,7 @@
       <c r="D221" s="2" t="n"/>
       <c r="E221" s="2" t="n"/>
       <c r="F221" s="2" t="n"/>
+      <c r="G221" s="2" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n"/>
@@ -2368,6 +2611,7 @@
       <c r="D222" s="2" t="n"/>
       <c r="E222" s="2" t="n"/>
       <c r="F222" s="2" t="n"/>
+      <c r="G222" s="2" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n"/>
@@ -2376,6 +2620,7 @@
       <c r="D223" s="2" t="n"/>
       <c r="E223" s="2" t="n"/>
       <c r="F223" s="2" t="n"/>
+      <c r="G223" s="2" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n"/>
@@ -2384,6 +2629,7 @@
       <c r="D224" s="2" t="n"/>
       <c r="E224" s="2" t="n"/>
       <c r="F224" s="2" t="n"/>
+      <c r="G224" s="2" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n"/>
@@ -2392,6 +2638,7 @@
       <c r="D225" s="2" t="n"/>
       <c r="E225" s="2" t="n"/>
       <c r="F225" s="2" t="n"/>
+      <c r="G225" s="2" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n"/>
@@ -2400,6 +2647,7 @@
       <c r="D226" s="2" t="n"/>
       <c r="E226" s="2" t="n"/>
       <c r="F226" s="2" t="n"/>
+      <c r="G226" s="2" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n"/>
@@ -2408,6 +2656,7 @@
       <c r="D227" s="2" t="n"/>
       <c r="E227" s="2" t="n"/>
       <c r="F227" s="2" t="n"/>
+      <c r="G227" s="2" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n"/>
@@ -2416,6 +2665,7 @@
       <c r="D228" s="2" t="n"/>
       <c r="E228" s="2" t="n"/>
       <c r="F228" s="2" t="n"/>
+      <c r="G228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n"/>
@@ -2424,6 +2674,7 @@
       <c r="D229" s="2" t="n"/>
       <c r="E229" s="2" t="n"/>
       <c r="F229" s="2" t="n"/>
+      <c r="G229" s="2" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n"/>
@@ -2432,6 +2683,7 @@
       <c r="D230" s="2" t="n"/>
       <c r="E230" s="2" t="n"/>
       <c r="F230" s="2" t="n"/>
+      <c r="G230" s="2" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n"/>
@@ -2440,6 +2692,7 @@
       <c r="D231" s="2" t="n"/>
       <c r="E231" s="2" t="n"/>
       <c r="F231" s="2" t="n"/>
+      <c r="G231" s="2" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n"/>
@@ -2448,6 +2701,7 @@
       <c r="D232" s="2" t="n"/>
       <c r="E232" s="2" t="n"/>
       <c r="F232" s="2" t="n"/>
+      <c r="G232" s="2" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n"/>
@@ -2456,6 +2710,7 @@
       <c r="D233" s="2" t="n"/>
       <c r="E233" s="2" t="n"/>
       <c r="F233" s="2" t="n"/>
+      <c r="G233" s="2" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n"/>
@@ -2464,6 +2719,7 @@
       <c r="D234" s="2" t="n"/>
       <c r="E234" s="2" t="n"/>
       <c r="F234" s="2" t="n"/>
+      <c r="G234" s="2" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n"/>
@@ -2472,6 +2728,7 @@
       <c r="D235" s="2" t="n"/>
       <c r="E235" s="2" t="n"/>
       <c r="F235" s="2" t="n"/>
+      <c r="G235" s="2" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n"/>
@@ -2480,6 +2737,7 @@
       <c r="D236" s="2" t="n"/>
       <c r="E236" s="2" t="n"/>
       <c r="F236" s="2" t="n"/>
+      <c r="G236" s="2" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n"/>
@@ -2488,6 +2746,7 @@
       <c r="D237" s="2" t="n"/>
       <c r="E237" s="2" t="n"/>
       <c r="F237" s="2" t="n"/>
+      <c r="G237" s="2" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n"/>
@@ -2496,6 +2755,7 @@
       <c r="D238" s="2" t="n"/>
       <c r="E238" s="2" t="n"/>
       <c r="F238" s="2" t="n"/>
+      <c r="G238" s="2" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n"/>
@@ -2504,6 +2764,7 @@
       <c r="D239" s="2" t="n"/>
       <c r="E239" s="2" t="n"/>
       <c r="F239" s="2" t="n"/>
+      <c r="G239" s="2" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n"/>
@@ -2512,6 +2773,7 @@
       <c r="D240" s="2" t="n"/>
       <c r="E240" s="2" t="n"/>
       <c r="F240" s="2" t="n"/>
+      <c r="G240" s="2" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n"/>
@@ -2520,6 +2782,7 @@
       <c r="D241" s="2" t="n"/>
       <c r="E241" s="2" t="n"/>
       <c r="F241" s="2" t="n"/>
+      <c r="G241" s="2" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n"/>
@@ -2528,6 +2791,7 @@
       <c r="D242" s="2" t="n"/>
       <c r="E242" s="2" t="n"/>
       <c r="F242" s="2" t="n"/>
+      <c r="G242" s="2" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n"/>
@@ -2536,6 +2800,7 @@
       <c r="D243" s="2" t="n"/>
       <c r="E243" s="2" t="n"/>
       <c r="F243" s="2" t="n"/>
+      <c r="G243" s="2" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n"/>
@@ -2544,6 +2809,7 @@
       <c r="D244" s="2" t="n"/>
       <c r="E244" s="2" t="n"/>
       <c r="F244" s="2" t="n"/>
+      <c r="G244" s="2" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n"/>
@@ -2552,6 +2818,7 @@
       <c r="D245" s="2" t="n"/>
       <c r="E245" s="2" t="n"/>
       <c r="F245" s="2" t="n"/>
+      <c r="G245" s="2" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n"/>
@@ -2560,6 +2827,7 @@
       <c r="D246" s="2" t="n"/>
       <c r="E246" s="2" t="n"/>
       <c r="F246" s="2" t="n"/>
+      <c r="G246" s="2" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n"/>
@@ -2568,6 +2836,7 @@
       <c r="D247" s="2" t="n"/>
       <c r="E247" s="2" t="n"/>
       <c r="F247" s="2" t="n"/>
+      <c r="G247" s="2" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n"/>
@@ -2576,6 +2845,7 @@
       <c r="D248" s="2" t="n"/>
       <c r="E248" s="2" t="n"/>
       <c r="F248" s="2" t="n"/>
+      <c r="G248" s="2" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n"/>
@@ -2584,6 +2854,7 @@
       <c r="D249" s="2" t="n"/>
       <c r="E249" s="2" t="n"/>
       <c r="F249" s="2" t="n"/>
+      <c r="G249" s="2" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n"/>
@@ -2592,6 +2863,7 @@
       <c r="D250" s="2" t="n"/>
       <c r="E250" s="2" t="n"/>
       <c r="F250" s="2" t="n"/>
+      <c r="G250" s="2" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n"/>
@@ -2600,6 +2872,7 @@
       <c r="D251" s="2" t="n"/>
       <c r="E251" s="2" t="n"/>
       <c r="F251" s="2" t="n"/>
+      <c r="G251" s="2" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n"/>
@@ -2608,6 +2881,7 @@
       <c r="D252" s="2" t="n"/>
       <c r="E252" s="2" t="n"/>
       <c r="F252" s="2" t="n"/>
+      <c r="G252" s="2" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n"/>
@@ -2616,6 +2890,7 @@
       <c r="D253" s="2" t="n"/>
       <c r="E253" s="2" t="n"/>
       <c r="F253" s="2" t="n"/>
+      <c r="G253" s="2" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n"/>
@@ -2624,6 +2899,7 @@
       <c r="D254" s="2" t="n"/>
       <c r="E254" s="2" t="n"/>
       <c r="F254" s="2" t="n"/>
+      <c r="G254" s="2" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n"/>
@@ -2632,6 +2908,7 @@
       <c r="D255" s="2" t="n"/>
       <c r="E255" s="2" t="n"/>
       <c r="F255" s="2" t="n"/>
+      <c r="G255" s="2" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n"/>
@@ -2640,6 +2917,7 @@
       <c r="D256" s="2" t="n"/>
       <c r="E256" s="2" t="n"/>
       <c r="F256" s="2" t="n"/>
+      <c r="G256" s="2" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n"/>
@@ -2648,6 +2926,7 @@
       <c r="D257" s="2" t="n"/>
       <c r="E257" s="2" t="n"/>
       <c r="F257" s="2" t="n"/>
+      <c r="G257" s="2" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n"/>
@@ -2656,6 +2935,7 @@
       <c r="D258" s="2" t="n"/>
       <c r="E258" s="2" t="n"/>
       <c r="F258" s="2" t="n"/>
+      <c r="G258" s="2" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n"/>
@@ -2664,6 +2944,7 @@
       <c r="D259" s="2" t="n"/>
       <c r="E259" s="2" t="n"/>
       <c r="F259" s="2" t="n"/>
+      <c r="G259" s="2" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n"/>
@@ -2672,6 +2953,7 @@
       <c r="D260" s="2" t="n"/>
       <c r="E260" s="2" t="n"/>
       <c r="F260" s="2" t="n"/>
+      <c r="G260" s="2" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n"/>
@@ -2680,6 +2962,7 @@
       <c r="D261" s="2" t="n"/>
       <c r="E261" s="2" t="n"/>
       <c r="F261" s="2" t="n"/>
+      <c r="G261" s="2" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n"/>
@@ -2688,6 +2971,7 @@
       <c r="D262" s="2" t="n"/>
       <c r="E262" s="2" t="n"/>
       <c r="F262" s="2" t="n"/>
+      <c r="G262" s="2" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n"/>
@@ -2696,6 +2980,7 @@
       <c r="D263" s="2" t="n"/>
       <c r="E263" s="2" t="n"/>
       <c r="F263" s="2" t="n"/>
+      <c r="G263" s="2" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="n"/>
@@ -2704,6 +2989,7 @@
       <c r="D264" s="2" t="n"/>
       <c r="E264" s="2" t="n"/>
       <c r="F264" s="2" t="n"/>
+      <c r="G264" s="2" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n"/>
@@ -2712,6 +2998,7 @@
       <c r="D265" s="2" t="n"/>
       <c r="E265" s="2" t="n"/>
       <c r="F265" s="2" t="n"/>
+      <c r="G265" s="2" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n"/>
@@ -2720,6 +3007,7 @@
       <c r="D266" s="2" t="n"/>
       <c r="E266" s="2" t="n"/>
       <c r="F266" s="2" t="n"/>
+      <c r="G266" s="2" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n"/>
@@ -2728,6 +3016,7 @@
       <c r="D267" s="2" t="n"/>
       <c r="E267" s="2" t="n"/>
       <c r="F267" s="2" t="n"/>
+      <c r="G267" s="2" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n"/>
@@ -2736,6 +3025,7 @@
       <c r="D268" s="2" t="n"/>
       <c r="E268" s="2" t="n"/>
       <c r="F268" s="2" t="n"/>
+      <c r="G268" s="2" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n"/>
@@ -2744,6 +3034,7 @@
       <c r="D269" s="2" t="n"/>
       <c r="E269" s="2" t="n"/>
       <c r="F269" s="2" t="n"/>
+      <c r="G269" s="2" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n"/>
@@ -2752,6 +3043,7 @@
       <c r="D270" s="2" t="n"/>
       <c r="E270" s="2" t="n"/>
       <c r="F270" s="2" t="n"/>
+      <c r="G270" s="2" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n"/>
@@ -2760,6 +3052,7 @@
       <c r="D271" s="2" t="n"/>
       <c r="E271" s="2" t="n"/>
       <c r="F271" s="2" t="n"/>
+      <c r="G271" s="2" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n"/>
@@ -2768,6 +3061,7 @@
       <c r="D272" s="2" t="n"/>
       <c r="E272" s="2" t="n"/>
       <c r="F272" s="2" t="n"/>
+      <c r="G272" s="2" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n"/>
@@ -2776,6 +3070,7 @@
       <c r="D273" s="2" t="n"/>
       <c r="E273" s="2" t="n"/>
       <c r="F273" s="2" t="n"/>
+      <c r="G273" s="2" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n"/>
@@ -2784,6 +3079,7 @@
       <c r="D274" s="2" t="n"/>
       <c r="E274" s="2" t="n"/>
       <c r="F274" s="2" t="n"/>
+      <c r="G274" s="2" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="n"/>
@@ -2792,6 +3088,7 @@
       <c r="D275" s="2" t="n"/>
       <c r="E275" s="2" t="n"/>
       <c r="F275" s="2" t="n"/>
+      <c r="G275" s="2" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n"/>
@@ -2800,6 +3097,7 @@
       <c r="D276" s="2" t="n"/>
       <c r="E276" s="2" t="n"/>
       <c r="F276" s="2" t="n"/>
+      <c r="G276" s="2" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n"/>
@@ -2808,6 +3106,7 @@
       <c r="D277" s="2" t="n"/>
       <c r="E277" s="2" t="n"/>
       <c r="F277" s="2" t="n"/>
+      <c r="G277" s="2" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n"/>
@@ -2816,6 +3115,7 @@
       <c r="D278" s="2" t="n"/>
       <c r="E278" s="2" t="n"/>
       <c r="F278" s="2" t="n"/>
+      <c r="G278" s="2" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n"/>
@@ -2824,6 +3124,7 @@
       <c r="D279" s="2" t="n"/>
       <c r="E279" s="2" t="n"/>
       <c r="F279" s="2" t="n"/>
+      <c r="G279" s="2" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n"/>
@@ -2832,6 +3133,7 @@
       <c r="D280" s="2" t="n"/>
       <c r="E280" s="2" t="n"/>
       <c r="F280" s="2" t="n"/>
+      <c r="G280" s="2" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n"/>
@@ -2840,6 +3142,7 @@
       <c r="D281" s="2" t="n"/>
       <c r="E281" s="2" t="n"/>
       <c r="F281" s="2" t="n"/>
+      <c r="G281" s="2" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="n"/>
@@ -2848,6 +3151,7 @@
       <c r="D282" s="2" t="n"/>
       <c r="E282" s="2" t="n"/>
       <c r="F282" s="2" t="n"/>
+      <c r="G282" s="2" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n"/>
@@ -2856,6 +3160,7 @@
       <c r="D283" s="2" t="n"/>
       <c r="E283" s="2" t="n"/>
       <c r="F283" s="2" t="n"/>
+      <c r="G283" s="2" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n"/>
@@ -2864,6 +3169,7 @@
       <c r="D284" s="2" t="n"/>
       <c r="E284" s="2" t="n"/>
       <c r="F284" s="2" t="n"/>
+      <c r="G284" s="2" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n"/>
@@ -2872,6 +3178,7 @@
       <c r="D285" s="2" t="n"/>
       <c r="E285" s="2" t="n"/>
       <c r="F285" s="2" t="n"/>
+      <c r="G285" s="2" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n"/>
@@ -2880,6 +3187,7 @@
       <c r="D286" s="2" t="n"/>
       <c r="E286" s="2" t="n"/>
       <c r="F286" s="2" t="n"/>
+      <c r="G286" s="2" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n"/>
@@ -2888,6 +3196,7 @@
       <c r="D287" s="2" t="n"/>
       <c r="E287" s="2" t="n"/>
       <c r="F287" s="2" t="n"/>
+      <c r="G287" s="2" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="n"/>
@@ -2896,6 +3205,7 @@
       <c r="D288" s="2" t="n"/>
       <c r="E288" s="2" t="n"/>
       <c r="F288" s="2" t="n"/>
+      <c r="G288" s="2" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n"/>
@@ -2904,6 +3214,7 @@
       <c r="D289" s="2" t="n"/>
       <c r="E289" s="2" t="n"/>
       <c r="F289" s="2" t="n"/>
+      <c r="G289" s="2" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n"/>
@@ -2912,6 +3223,7 @@
       <c r="D290" s="2" t="n"/>
       <c r="E290" s="2" t="n"/>
       <c r="F290" s="2" t="n"/>
+      <c r="G290" s="2" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n"/>
@@ -2920,6 +3232,7 @@
       <c r="D291" s="2" t="n"/>
       <c r="E291" s="2" t="n"/>
       <c r="F291" s="2" t="n"/>
+      <c r="G291" s="2" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n"/>
@@ -2928,6 +3241,7 @@
       <c r="D292" s="2" t="n"/>
       <c r="E292" s="2" t="n"/>
       <c r="F292" s="2" t="n"/>
+      <c r="G292" s="2" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n"/>
@@ -2936,6 +3250,7 @@
       <c r="D293" s="2" t="n"/>
       <c r="E293" s="2" t="n"/>
       <c r="F293" s="2" t="n"/>
+      <c r="G293" s="2" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n"/>
@@ -2944,6 +3259,7 @@
       <c r="D294" s="2" t="n"/>
       <c r="E294" s="2" t="n"/>
       <c r="F294" s="2" t="n"/>
+      <c r="G294" s="2" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="n"/>
@@ -2952,6 +3268,7 @@
       <c r="D295" s="2" t="n"/>
       <c r="E295" s="2" t="n"/>
       <c r="F295" s="2" t="n"/>
+      <c r="G295" s="2" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n"/>
@@ -2960,6 +3277,7 @@
       <c r="D296" s="2" t="n"/>
       <c r="E296" s="2" t="n"/>
       <c r="F296" s="2" t="n"/>
+      <c r="G296" s="2" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n"/>
@@ -2968,6 +3286,7 @@
       <c r="D297" s="2" t="n"/>
       <c r="E297" s="2" t="n"/>
       <c r="F297" s="2" t="n"/>
+      <c r="G297" s="2" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n"/>
@@ -2976,6 +3295,7 @@
       <c r="D298" s="2" t="n"/>
       <c r="E298" s="2" t="n"/>
       <c r="F298" s="2" t="n"/>
+      <c r="G298" s="2" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n"/>
@@ -2984,6 +3304,7 @@
       <c r="D299" s="2" t="n"/>
       <c r="E299" s="2" t="n"/>
       <c r="F299" s="2" t="n"/>
+      <c r="G299" s="2" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n"/>
@@ -2992,6 +3313,7 @@
       <c r="D300" s="2" t="n"/>
       <c r="E300" s="2" t="n"/>
       <c r="F300" s="2" t="n"/>
+      <c r="G300" s="2" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="n"/>
@@ -3000,6 +3322,7 @@
       <c r="D301" s="2" t="n"/>
       <c r="E301" s="2" t="n"/>
       <c r="F301" s="2" t="n"/>
+      <c r="G301" s="2" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="2" t="n"/>
@@ -3008,6 +3331,7 @@
       <c r="D302" s="2" t="n"/>
       <c r="E302" s="2" t="n"/>
       <c r="F302" s="2" t="n"/>
+      <c r="G302" s="2" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="2" t="n"/>
@@ -3016,6 +3340,7 @@
       <c r="D303" s="2" t="n"/>
       <c r="E303" s="2" t="n"/>
       <c r="F303" s="2" t="n"/>
+      <c r="G303" s="2" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="n"/>
@@ -3024,6 +3349,7 @@
       <c r="D304" s="2" t="n"/>
       <c r="E304" s="2" t="n"/>
       <c r="F304" s="2" t="n"/>
+      <c r="G304" s="2" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="n"/>
@@ -3032,6 +3358,7 @@
       <c r="D305" s="2" t="n"/>
       <c r="E305" s="2" t="n"/>
       <c r="F305" s="2" t="n"/>
+      <c r="G305" s="2" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="n"/>
@@ -3040,6 +3367,7 @@
       <c r="D306" s="2" t="n"/>
       <c r="E306" s="2" t="n"/>
       <c r="F306" s="2" t="n"/>
+      <c r="G306" s="2" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="n"/>
@@ -3048,6 +3376,7 @@
       <c r="D307" s="2" t="n"/>
       <c r="E307" s="2" t="n"/>
       <c r="F307" s="2" t="n"/>
+      <c r="G307" s="2" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="n"/>
@@ -3056,6 +3385,7 @@
       <c r="D308" s="2" t="n"/>
       <c r="E308" s="2" t="n"/>
       <c r="F308" s="2" t="n"/>
+      <c r="G308" s="2" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="2" t="n"/>
@@ -3064,6 +3394,7 @@
       <c r="D309" s="2" t="n"/>
       <c r="E309" s="2" t="n"/>
       <c r="F309" s="2" t="n"/>
+      <c r="G309" s="2" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="n"/>
@@ -3072,6 +3403,7 @@
       <c r="D310" s="2" t="n"/>
       <c r="E310" s="2" t="n"/>
       <c r="F310" s="2" t="n"/>
+      <c r="G310" s="2" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="2" t="n"/>
@@ -3080,6 +3412,7 @@
       <c r="D311" s="2" t="n"/>
       <c r="E311" s="2" t="n"/>
       <c r="F311" s="2" t="n"/>
+      <c r="G311" s="2" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="n"/>
@@ -3088,6 +3421,7 @@
       <c r="D312" s="2" t="n"/>
       <c r="E312" s="2" t="n"/>
       <c r="F312" s="2" t="n"/>
+      <c r="G312" s="2" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="2" t="n"/>
@@ -3096,6 +3430,7 @@
       <c r="D313" s="2" t="n"/>
       <c r="E313" s="2" t="n"/>
       <c r="F313" s="2" t="n"/>
+      <c r="G313" s="2" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="n"/>
@@ -3104,6 +3439,7 @@
       <c r="D314" s="2" t="n"/>
       <c r="E314" s="2" t="n"/>
       <c r="F314" s="2" t="n"/>
+      <c r="G314" s="2" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="2" t="n"/>
@@ -3112,6 +3448,7 @@
       <c r="D315" s="2" t="n"/>
       <c r="E315" s="2" t="n"/>
       <c r="F315" s="2" t="n"/>
+      <c r="G315" s="2" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="n"/>
@@ -3120,6 +3457,7 @@
       <c r="D316" s="2" t="n"/>
       <c r="E316" s="2" t="n"/>
       <c r="F316" s="2" t="n"/>
+      <c r="G316" s="2" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="2" t="n"/>
@@ -3128,6 +3466,7 @@
       <c r="D317" s="2" t="n"/>
       <c r="E317" s="2" t="n"/>
       <c r="F317" s="2" t="n"/>
+      <c r="G317" s="2" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="n"/>
@@ -3136,6 +3475,7 @@
       <c r="D318" s="2" t="n"/>
       <c r="E318" s="2" t="n"/>
       <c r="F318" s="2" t="n"/>
+      <c r="G318" s="2" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="2" t="n"/>
@@ -3144,6 +3484,7 @@
       <c r="D319" s="2" t="n"/>
       <c r="E319" s="2" t="n"/>
       <c r="F319" s="2" t="n"/>
+      <c r="G319" s="2" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="n"/>
@@ -3152,6 +3493,7 @@
       <c r="D320" s="2" t="n"/>
       <c r="E320" s="2" t="n"/>
       <c r="F320" s="2" t="n"/>
+      <c r="G320" s="2" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="2" t="n"/>
@@ -3160,6 +3502,7 @@
       <c r="D321" s="2" t="n"/>
       <c r="E321" s="2" t="n"/>
       <c r="F321" s="2" t="n"/>
+      <c r="G321" s="2" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="n"/>
@@ -3168,6 +3511,7 @@
       <c r="D322" s="2" t="n"/>
       <c r="E322" s="2" t="n"/>
       <c r="F322" s="2" t="n"/>
+      <c r="G322" s="2" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="n"/>
@@ -3176,6 +3520,7 @@
       <c r="D323" s="2" t="n"/>
       <c r="E323" s="2" t="n"/>
       <c r="F323" s="2" t="n"/>
+      <c r="G323" s="2" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="2" t="n"/>
@@ -3184,6 +3529,7 @@
       <c r="D324" s="2" t="n"/>
       <c r="E324" s="2" t="n"/>
       <c r="F324" s="2" t="n"/>
+      <c r="G324" s="2" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="2" t="n"/>
@@ -3192,6 +3538,7 @@
       <c r="D325" s="2" t="n"/>
       <c r="E325" s="2" t="n"/>
       <c r="F325" s="2" t="n"/>
+      <c r="G325" s="2" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="2" t="n"/>
@@ -3200,6 +3547,7 @@
       <c r="D326" s="2" t="n"/>
       <c r="E326" s="2" t="n"/>
       <c r="F326" s="2" t="n"/>
+      <c r="G326" s="2" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="2" t="n"/>
@@ -3208,6 +3556,7 @@
       <c r="D327" s="2" t="n"/>
       <c r="E327" s="2" t="n"/>
       <c r="F327" s="2" t="n"/>
+      <c r="G327" s="2" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="2" t="n"/>
@@ -3216,6 +3565,7 @@
       <c r="D328" s="2" t="n"/>
       <c r="E328" s="2" t="n"/>
       <c r="F328" s="2" t="n"/>
+      <c r="G328" s="2" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="2" t="n"/>
@@ -3224,6 +3574,7 @@
       <c r="D329" s="2" t="n"/>
       <c r="E329" s="2" t="n"/>
       <c r="F329" s="2" t="n"/>
+      <c r="G329" s="2" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="2" t="n"/>
@@ -3232,6 +3583,7 @@
       <c r="D330" s="2" t="n"/>
       <c r="E330" s="2" t="n"/>
       <c r="F330" s="2" t="n"/>
+      <c r="G330" s="2" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="2" t="n"/>
@@ -3240,6 +3592,7 @@
       <c r="D331" s="2" t="n"/>
       <c r="E331" s="2" t="n"/>
       <c r="F331" s="2" t="n"/>
+      <c r="G331" s="2" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="2" t="n"/>
@@ -3248,6 +3601,7 @@
       <c r="D332" s="2" t="n"/>
       <c r="E332" s="2" t="n"/>
       <c r="F332" s="2" t="n"/>
+      <c r="G332" s="2" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="2" t="n"/>
@@ -3256,6 +3610,7 @@
       <c r="D333" s="2" t="n"/>
       <c r="E333" s="2" t="n"/>
       <c r="F333" s="2" t="n"/>
+      <c r="G333" s="2" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="2" t="n"/>
@@ -3264,6 +3619,7 @@
       <c r="D334" s="2" t="n"/>
       <c r="E334" s="2" t="n"/>
       <c r="F334" s="2" t="n"/>
+      <c r="G334" s="2" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="n"/>
@@ -3272,6 +3628,7 @@
       <c r="D335" s="2" t="n"/>
       <c r="E335" s="2" t="n"/>
       <c r="F335" s="2" t="n"/>
+      <c r="G335" s="2" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="2" t="n"/>
@@ -3280,6 +3637,7 @@
       <c r="D336" s="2" t="n"/>
       <c r="E336" s="2" t="n"/>
       <c r="F336" s="2" t="n"/>
+      <c r="G336" s="2" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="n"/>
@@ -3288,6 +3646,7 @@
       <c r="D337" s="2" t="n"/>
       <c r="E337" s="2" t="n"/>
       <c r="F337" s="2" t="n"/>
+      <c r="G337" s="2" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="n"/>
@@ -3296,6 +3655,7 @@
       <c r="D338" s="2" t="n"/>
       <c r="E338" s="2" t="n"/>
       <c r="F338" s="2" t="n"/>
+      <c r="G338" s="2" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="n"/>
@@ -3304,6 +3664,7 @@
       <c r="D339" s="2" t="n"/>
       <c r="E339" s="2" t="n"/>
       <c r="F339" s="2" t="n"/>
+      <c r="G339" s="2" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="2" t="n"/>
@@ -3312,6 +3673,7 @@
       <c r="D340" s="2" t="n"/>
       <c r="E340" s="2" t="n"/>
       <c r="F340" s="2" t="n"/>
+      <c r="G340" s="2" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="2" t="n"/>
@@ -3320,6 +3682,7 @@
       <c r="D341" s="2" t="n"/>
       <c r="E341" s="2" t="n"/>
       <c r="F341" s="2" t="n"/>
+      <c r="G341" s="2" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="2" t="n"/>
@@ -3328,6 +3691,7 @@
       <c r="D342" s="2" t="n"/>
       <c r="E342" s="2" t="n"/>
       <c r="F342" s="2" t="n"/>
+      <c r="G342" s="2" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="n"/>
@@ -3336,6 +3700,7 @@
       <c r="D343" s="2" t="n"/>
       <c r="E343" s="2" t="n"/>
       <c r="F343" s="2" t="n"/>
+      <c r="G343" s="2" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="2" t="n"/>
@@ -3344,6 +3709,7 @@
       <c r="D344" s="2" t="n"/>
       <c r="E344" s="2" t="n"/>
       <c r="F344" s="2" t="n"/>
+      <c r="G344" s="2" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="2" t="n"/>
@@ -3352,6 +3718,7 @@
       <c r="D345" s="2" t="n"/>
       <c r="E345" s="2" t="n"/>
       <c r="F345" s="2" t="n"/>
+      <c r="G345" s="2" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="2" t="n"/>
@@ -3360,6 +3727,7 @@
       <c r="D346" s="2" t="n"/>
       <c r="E346" s="2" t="n"/>
       <c r="F346" s="2" t="n"/>
+      <c r="G346" s="2" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="2" t="n"/>
@@ -3368,6 +3736,7 @@
       <c r="D347" s="2" t="n"/>
       <c r="E347" s="2" t="n"/>
       <c r="F347" s="2" t="n"/>
+      <c r="G347" s="2" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="2" t="n"/>
@@ -3376,6 +3745,7 @@
       <c r="D348" s="2" t="n"/>
       <c r="E348" s="2" t="n"/>
       <c r="F348" s="2" t="n"/>
+      <c r="G348" s="2" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="n"/>
@@ -3384,6 +3754,7 @@
       <c r="D349" s="2" t="n"/>
       <c r="E349" s="2" t="n"/>
       <c r="F349" s="2" t="n"/>
+      <c r="G349" s="2" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="2" t="n"/>
@@ -3392,6 +3763,7 @@
       <c r="D350" s="2" t="n"/>
       <c r="E350" s="2" t="n"/>
       <c r="F350" s="2" t="n"/>
+      <c r="G350" s="2" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="n"/>
@@ -3400,6 +3772,7 @@
       <c r="D351" s="2" t="n"/>
       <c r="E351" s="2" t="n"/>
       <c r="F351" s="2" t="n"/>
+      <c r="G351" s="2" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="2" t="n"/>
@@ -3408,6 +3781,7 @@
       <c r="D352" s="2" t="n"/>
       <c r="E352" s="2" t="n"/>
       <c r="F352" s="2" t="n"/>
+      <c r="G352" s="2" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="2" t="n"/>
@@ -3416,6 +3790,7 @@
       <c r="D353" s="2" t="n"/>
       <c r="E353" s="2" t="n"/>
       <c r="F353" s="2" t="n"/>
+      <c r="G353" s="2" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="2" t="n"/>
@@ -3424,6 +3799,7 @@
       <c r="D354" s="2" t="n"/>
       <c r="E354" s="2" t="n"/>
       <c r="F354" s="2" t="n"/>
+      <c r="G354" s="2" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="2" t="n"/>
@@ -3432,6 +3808,7 @@
       <c r="D355" s="2" t="n"/>
       <c r="E355" s="2" t="n"/>
       <c r="F355" s="2" t="n"/>
+      <c r="G355" s="2" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="2" t="n"/>
@@ -3440,6 +3817,7 @@
       <c r="D356" s="2" t="n"/>
       <c r="E356" s="2" t="n"/>
       <c r="F356" s="2" t="n"/>
+      <c r="G356" s="2" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="n"/>
@@ -3448,6 +3826,7 @@
       <c r="D357" s="2" t="n"/>
       <c r="E357" s="2" t="n"/>
       <c r="F357" s="2" t="n"/>
+      <c r="G357" s="2" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="2" t="n"/>
@@ -3456,6 +3835,7 @@
       <c r="D358" s="2" t="n"/>
       <c r="E358" s="2" t="n"/>
       <c r="F358" s="2" t="n"/>
+      <c r="G358" s="2" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="n"/>
@@ -3464,6 +3844,7 @@
       <c r="D359" s="2" t="n"/>
       <c r="E359" s="2" t="n"/>
       <c r="F359" s="2" t="n"/>
+      <c r="G359" s="2" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="2" t="n"/>
@@ -3472,6 +3853,7 @@
       <c r="D360" s="2" t="n"/>
       <c r="E360" s="2" t="n"/>
       <c r="F360" s="2" t="n"/>
+      <c r="G360" s="2" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="2" t="n"/>
@@ -3480,6 +3862,7 @@
       <c r="D361" s="2" t="n"/>
       <c r="E361" s="2" t="n"/>
       <c r="F361" s="2" t="n"/>
+      <c r="G361" s="2" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="n"/>
@@ -3488,6 +3871,7 @@
       <c r="D362" s="2" t="n"/>
       <c r="E362" s="2" t="n"/>
       <c r="F362" s="2" t="n"/>
+      <c r="G362" s="2" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="2" t="n"/>
@@ -3496,6 +3880,7 @@
       <c r="D363" s="2" t="n"/>
       <c r="E363" s="2" t="n"/>
       <c r="F363" s="2" t="n"/>
+      <c r="G363" s="2" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="2" t="n"/>
@@ -3504,6 +3889,7 @@
       <c r="D364" s="2" t="n"/>
       <c r="E364" s="2" t="n"/>
       <c r="F364" s="2" t="n"/>
+      <c r="G364" s="2" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="2" t="n"/>
@@ -3512,6 +3898,7 @@
       <c r="D365" s="2" t="n"/>
       <c r="E365" s="2" t="n"/>
       <c r="F365" s="2" t="n"/>
+      <c r="G365" s="2" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="2" t="n"/>
@@ -3520,6 +3907,7 @@
       <c r="D366" s="2" t="n"/>
       <c r="E366" s="2" t="n"/>
       <c r="F366" s="2" t="n"/>
+      <c r="G366" s="2" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="2" t="n"/>
@@ -3528,6 +3916,7 @@
       <c r="D367" s="2" t="n"/>
       <c r="E367" s="2" t="n"/>
       <c r="F367" s="2" t="n"/>
+      <c r="G367" s="2" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="n"/>
@@ -3536,6 +3925,7 @@
       <c r="D368" s="2" t="n"/>
       <c r="E368" s="2" t="n"/>
       <c r="F368" s="2" t="n"/>
+      <c r="G368" s="2" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="2" t="n"/>
@@ -3544,6 +3934,7 @@
       <c r="D369" s="2" t="n"/>
       <c r="E369" s="2" t="n"/>
       <c r="F369" s="2" t="n"/>
+      <c r="G369" s="2" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="2" t="n"/>
@@ -3552,6 +3943,7 @@
       <c r="D370" s="2" t="n"/>
       <c r="E370" s="2" t="n"/>
       <c r="F370" s="2" t="n"/>
+      <c r="G370" s="2" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="n"/>
@@ -3560,6 +3952,7 @@
       <c r="D371" s="2" t="n"/>
       <c r="E371" s="2" t="n"/>
       <c r="F371" s="2" t="n"/>
+      <c r="G371" s="2" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="2" t="n"/>
@@ -3568,6 +3961,7 @@
       <c r="D372" s="2" t="n"/>
       <c r="E372" s="2" t="n"/>
       <c r="F372" s="2" t="n"/>
+      <c r="G372" s="2" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="2" t="n"/>
@@ -3576,6 +3970,7 @@
       <c r="D373" s="2" t="n"/>
       <c r="E373" s="2" t="n"/>
       <c r="F373" s="2" t="n"/>
+      <c r="G373" s="2" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="n"/>
@@ -3584,6 +3979,7 @@
       <c r="D374" s="2" t="n"/>
       <c r="E374" s="2" t="n"/>
       <c r="F374" s="2" t="n"/>
+      <c r="G374" s="2" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="n"/>
@@ -3592,6 +3988,7 @@
       <c r="D375" s="2" t="n"/>
       <c r="E375" s="2" t="n"/>
       <c r="F375" s="2" t="n"/>
+      <c r="G375" s="2" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="n"/>
@@ -3600,6 +3997,7 @@
       <c r="D376" s="2" t="n"/>
       <c r="E376" s="2" t="n"/>
       <c r="F376" s="2" t="n"/>
+      <c r="G376" s="2" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="2" t="n"/>
@@ -3608,6 +4006,7 @@
       <c r="D377" s="2" t="n"/>
       <c r="E377" s="2" t="n"/>
       <c r="F377" s="2" t="n"/>
+      <c r="G377" s="2" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="2" t="n"/>
@@ -3616,6 +4015,7 @@
       <c r="D378" s="2" t="n"/>
       <c r="E378" s="2" t="n"/>
       <c r="F378" s="2" t="n"/>
+      <c r="G378" s="2" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="2" t="n"/>
@@ -3624,6 +4024,7 @@
       <c r="D379" s="2" t="n"/>
       <c r="E379" s="2" t="n"/>
       <c r="F379" s="2" t="n"/>
+      <c r="G379" s="2" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="2" t="n"/>
@@ -3632,6 +4033,7 @@
       <c r="D380" s="2" t="n"/>
       <c r="E380" s="2" t="n"/>
       <c r="F380" s="2" t="n"/>
+      <c r="G380" s="2" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="2" t="n"/>
@@ -3640,6 +4042,7 @@
       <c r="D381" s="2" t="n"/>
       <c r="E381" s="2" t="n"/>
       <c r="F381" s="2" t="n"/>
+      <c r="G381" s="2" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="2" t="n"/>
@@ -3648,6 +4051,7 @@
       <c r="D382" s="2" t="n"/>
       <c r="E382" s="2" t="n"/>
       <c r="F382" s="2" t="n"/>
+      <c r="G382" s="2" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="2" t="n"/>
@@ -3656,6 +4060,7 @@
       <c r="D383" s="2" t="n"/>
       <c r="E383" s="2" t="n"/>
       <c r="F383" s="2" t="n"/>
+      <c r="G383" s="2" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="2" t="n"/>
@@ -3664,6 +4069,7 @@
       <c r="D384" s="2" t="n"/>
       <c r="E384" s="2" t="n"/>
       <c r="F384" s="2" t="n"/>
+      <c r="G384" s="2" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="2" t="n"/>
@@ -3672,6 +4078,7 @@
       <c r="D385" s="2" t="n"/>
       <c r="E385" s="2" t="n"/>
       <c r="F385" s="2" t="n"/>
+      <c r="G385" s="2" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="n"/>
@@ -3680,6 +4087,7 @@
       <c r="D386" s="2" t="n"/>
       <c r="E386" s="2" t="n"/>
       <c r="F386" s="2" t="n"/>
+      <c r="G386" s="2" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="2" t="n"/>
@@ -3688,6 +4096,7 @@
       <c r="D387" s="2" t="n"/>
       <c r="E387" s="2" t="n"/>
       <c r="F387" s="2" t="n"/>
+      <c r="G387" s="2" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="2" t="n"/>
@@ -3696,6 +4105,7 @@
       <c r="D388" s="2" t="n"/>
       <c r="E388" s="2" t="n"/>
       <c r="F388" s="2" t="n"/>
+      <c r="G388" s="2" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="2" t="n"/>
@@ -3704,6 +4114,7 @@
       <c r="D389" s="2" t="n"/>
       <c r="E389" s="2" t="n"/>
       <c r="F389" s="2" t="n"/>
+      <c r="G389" s="2" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="2" t="n"/>
@@ -3712,6 +4123,7 @@
       <c r="D390" s="2" t="n"/>
       <c r="E390" s="2" t="n"/>
       <c r="F390" s="2" t="n"/>
+      <c r="G390" s="2" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="2" t="n"/>
@@ -3720,6 +4132,7 @@
       <c r="D391" s="2" t="n"/>
       <c r="E391" s="2" t="n"/>
       <c r="F391" s="2" t="n"/>
+      <c r="G391" s="2" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="2" t="n"/>
@@ -3728,6 +4141,7 @@
       <c r="D392" s="2" t="n"/>
       <c r="E392" s="2" t="n"/>
       <c r="F392" s="2" t="n"/>
+      <c r="G392" s="2" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="2" t="n"/>
@@ -3736,6 +4150,7 @@
       <c r="D393" s="2" t="n"/>
       <c r="E393" s="2" t="n"/>
       <c r="F393" s="2" t="n"/>
+      <c r="G393" s="2" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="2" t="n"/>
@@ -3744,6 +4159,7 @@
       <c r="D394" s="2" t="n"/>
       <c r="E394" s="2" t="n"/>
       <c r="F394" s="2" t="n"/>
+      <c r="G394" s="2" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="2" t="n"/>
@@ -3752,6 +4168,7 @@
       <c r="D395" s="2" t="n"/>
       <c r="E395" s="2" t="n"/>
       <c r="F395" s="2" t="n"/>
+      <c r="G395" s="2" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="2" t="n"/>
@@ -3760,6 +4177,7 @@
       <c r="D396" s="2" t="n"/>
       <c r="E396" s="2" t="n"/>
       <c r="F396" s="2" t="n"/>
+      <c r="G396" s="2" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="2" t="n"/>
@@ -3768,6 +4186,7 @@
       <c r="D397" s="2" t="n"/>
       <c r="E397" s="2" t="n"/>
       <c r="F397" s="2" t="n"/>
+      <c r="G397" s="2" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="2" t="n"/>
@@ -3776,6 +4195,7 @@
       <c r="D398" s="2" t="n"/>
       <c r="E398" s="2" t="n"/>
       <c r="F398" s="2" t="n"/>
+      <c r="G398" s="2" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="n"/>
@@ -3784,6 +4204,7 @@
       <c r="D399" s="2" t="n"/>
       <c r="E399" s="2" t="n"/>
       <c r="F399" s="2" t="n"/>
+      <c r="G399" s="2" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="2" t="n"/>
@@ -3792,6 +4213,7 @@
       <c r="D400" s="2" t="n"/>
       <c r="E400" s="2" t="n"/>
       <c r="F400" s="2" t="n"/>
+      <c r="G400" s="2" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="2" t="n"/>
@@ -3800,6 +4222,7 @@
       <c r="D401" s="2" t="n"/>
       <c r="E401" s="2" t="n"/>
       <c r="F401" s="2" t="n"/>
+      <c r="G401" s="2" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="2" t="n"/>
@@ -3808,6 +4231,7 @@
       <c r="D402" s="2" t="n"/>
       <c r="E402" s="2" t="n"/>
       <c r="F402" s="2" t="n"/>
+      <c r="G402" s="2" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="2" t="n"/>
@@ -3816,6 +4240,7 @@
       <c r="D403" s="2" t="n"/>
       <c r="E403" s="2" t="n"/>
       <c r="F403" s="2" t="n"/>
+      <c r="G403" s="2" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="2" t="n"/>
@@ -3824,6 +4249,7 @@
       <c r="D404" s="2" t="n"/>
       <c r="E404" s="2" t="n"/>
       <c r="F404" s="2" t="n"/>
+      <c r="G404" s="2" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="2" t="n"/>
@@ -3832,6 +4258,7 @@
       <c r="D405" s="2" t="n"/>
       <c r="E405" s="2" t="n"/>
       <c r="F405" s="2" t="n"/>
+      <c r="G405" s="2" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="2" t="n"/>
@@ -3840,6 +4267,7 @@
       <c r="D406" s="2" t="n"/>
       <c r="E406" s="2" t="n"/>
       <c r="F406" s="2" t="n"/>
+      <c r="G406" s="2" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="2" t="n"/>
@@ -3848,6 +4276,7 @@
       <c r="D407" s="2" t="n"/>
       <c r="E407" s="2" t="n"/>
       <c r="F407" s="2" t="n"/>
+      <c r="G407" s="2" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n"/>
@@ -3856,6 +4285,7 @@
       <c r="D408" s="2" t="n"/>
       <c r="E408" s="2" t="n"/>
       <c r="F408" s="2" t="n"/>
+      <c r="G408" s="2" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n"/>
@@ -3864,6 +4294,7 @@
       <c r="D409" s="2" t="n"/>
       <c r="E409" s="2" t="n"/>
       <c r="F409" s="2" t="n"/>
+      <c r="G409" s="2" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n"/>
@@ -3872,6 +4303,7 @@
       <c r="D410" s="2" t="n"/>
       <c r="E410" s="2" t="n"/>
       <c r="F410" s="2" t="n"/>
+      <c r="G410" s="2" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="2" t="n"/>
@@ -3880,6 +4312,7 @@
       <c r="D411" s="2" t="n"/>
       <c r="E411" s="2" t="n"/>
       <c r="F411" s="2" t="n"/>
+      <c r="G411" s="2" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="2" t="n"/>
@@ -3888,6 +4321,7 @@
       <c r="D412" s="2" t="n"/>
       <c r="E412" s="2" t="n"/>
       <c r="F412" s="2" t="n"/>
+      <c r="G412" s="2" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="2" t="n"/>
@@ -3896,6 +4330,7 @@
       <c r="D413" s="2" t="n"/>
       <c r="E413" s="2" t="n"/>
       <c r="F413" s="2" t="n"/>
+      <c r="G413" s="2" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="2" t="n"/>
@@ -3904,6 +4339,7 @@
       <c r="D414" s="2" t="n"/>
       <c r="E414" s="2" t="n"/>
       <c r="F414" s="2" t="n"/>
+      <c r="G414" s="2" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="2" t="n"/>
@@ -3912,6 +4348,7 @@
       <c r="D415" s="2" t="n"/>
       <c r="E415" s="2" t="n"/>
       <c r="F415" s="2" t="n"/>
+      <c r="G415" s="2" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="2" t="n"/>
@@ -3920,6 +4357,7 @@
       <c r="D416" s="2" t="n"/>
       <c r="E416" s="2" t="n"/>
       <c r="F416" s="2" t="n"/>
+      <c r="G416" s="2" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="2" t="n"/>
@@ -3928,6 +4366,7 @@
       <c r="D417" s="2" t="n"/>
       <c r="E417" s="2" t="n"/>
       <c r="F417" s="2" t="n"/>
+      <c r="G417" s="2" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="2" t="n"/>
@@ -3936,6 +4375,7 @@
       <c r="D418" s="2" t="n"/>
       <c r="E418" s="2" t="n"/>
       <c r="F418" s="2" t="n"/>
+      <c r="G418" s="2" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="2" t="n"/>
@@ -3944,6 +4384,7 @@
       <c r="D419" s="2" t="n"/>
       <c r="E419" s="2" t="n"/>
       <c r="F419" s="2" t="n"/>
+      <c r="G419" s="2" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="2" t="n"/>
@@ -3952,6 +4393,7 @@
       <c r="D420" s="2" t="n"/>
       <c r="E420" s="2" t="n"/>
       <c r="F420" s="2" t="n"/>
+      <c r="G420" s="2" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="2" t="n"/>
@@ -3960,6 +4402,7 @@
       <c r="D421" s="2" t="n"/>
       <c r="E421" s="2" t="n"/>
       <c r="F421" s="2" t="n"/>
+      <c r="G421" s="2" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="2" t="n"/>
@@ -3968,6 +4411,7 @@
       <c r="D422" s="2" t="n"/>
       <c r="E422" s="2" t="n"/>
       <c r="F422" s="2" t="n"/>
+      <c r="G422" s="2" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="2" t="n"/>
@@ -3976,6 +4420,7 @@
       <c r="D423" s="2" t="n"/>
       <c r="E423" s="2" t="n"/>
       <c r="F423" s="2" t="n"/>
+      <c r="G423" s="2" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="2" t="n"/>
@@ -3984,6 +4429,7 @@
       <c r="D424" s="2" t="n"/>
       <c r="E424" s="2" t="n"/>
       <c r="F424" s="2" t="n"/>
+      <c r="G424" s="2" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="2" t="n"/>
@@ -3992,6 +4438,7 @@
       <c r="D425" s="2" t="n"/>
       <c r="E425" s="2" t="n"/>
       <c r="F425" s="2" t="n"/>
+      <c r="G425" s="2" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="2" t="n"/>
@@ -4000,6 +4447,7 @@
       <c r="D426" s="2" t="n"/>
       <c r="E426" s="2" t="n"/>
       <c r="F426" s="2" t="n"/>
+      <c r="G426" s="2" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="2" t="n"/>
@@ -4008,6 +4456,7 @@
       <c r="D427" s="2" t="n"/>
       <c r="E427" s="2" t="n"/>
       <c r="F427" s="2" t="n"/>
+      <c r="G427" s="2" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="2" t="n"/>
@@ -4016,6 +4465,7 @@
       <c r="D428" s="2" t="n"/>
       <c r="E428" s="2" t="n"/>
       <c r="F428" s="2" t="n"/>
+      <c r="G428" s="2" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="2" t="n"/>
@@ -4024,6 +4474,7 @@
       <c r="D429" s="2" t="n"/>
       <c r="E429" s="2" t="n"/>
       <c r="F429" s="2" t="n"/>
+      <c r="G429" s="2" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="2" t="n"/>
@@ -4032,6 +4483,7 @@
       <c r="D430" s="2" t="n"/>
       <c r="E430" s="2" t="n"/>
       <c r="F430" s="2" t="n"/>
+      <c r="G430" s="2" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="2" t="n"/>
@@ -4040,6 +4492,7 @@
       <c r="D431" s="2" t="n"/>
       <c r="E431" s="2" t="n"/>
       <c r="F431" s="2" t="n"/>
+      <c r="G431" s="2" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="2" t="n"/>
@@ -4048,6 +4501,7 @@
       <c r="D432" s="2" t="n"/>
       <c r="E432" s="2" t="n"/>
       <c r="F432" s="2" t="n"/>
+      <c r="G432" s="2" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="2" t="n"/>
@@ -4056,6 +4510,7 @@
       <c r="D433" s="2" t="n"/>
       <c r="E433" s="2" t="n"/>
       <c r="F433" s="2" t="n"/>
+      <c r="G433" s="2" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="2" t="n"/>
@@ -4064,6 +4519,7 @@
       <c r="D434" s="2" t="n"/>
       <c r="E434" s="2" t="n"/>
       <c r="F434" s="2" t="n"/>
+      <c r="G434" s="2" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n"/>
@@ -4072,6 +4528,7 @@
       <c r="D435" s="2" t="n"/>
       <c r="E435" s="2" t="n"/>
       <c r="F435" s="2" t="n"/>
+      <c r="G435" s="2" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n"/>
@@ -4080,6 +4537,7 @@
       <c r="D436" s="2" t="n"/>
       <c r="E436" s="2" t="n"/>
       <c r="F436" s="2" t="n"/>
+      <c r="G436" s="2" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="2" t="n"/>
@@ -4088,6 +4546,7 @@
       <c r="D437" s="2" t="n"/>
       <c r="E437" s="2" t="n"/>
       <c r="F437" s="2" t="n"/>
+      <c r="G437" s="2" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="2" t="n"/>
@@ -4096,6 +4555,7 @@
       <c r="D438" s="2" t="n"/>
       <c r="E438" s="2" t="n"/>
       <c r="F438" s="2" t="n"/>
+      <c r="G438" s="2" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="2" t="n"/>
@@ -4104,6 +4564,7 @@
       <c r="D439" s="2" t="n"/>
       <c r="E439" s="2" t="n"/>
       <c r="F439" s="2" t="n"/>
+      <c r="G439" s="2" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="2" t="n"/>
@@ -4112,6 +4573,7 @@
       <c r="D440" s="2" t="n"/>
       <c r="E440" s="2" t="n"/>
       <c r="F440" s="2" t="n"/>
+      <c r="G440" s="2" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="2" t="n"/>
@@ -4120,6 +4582,7 @@
       <c r="D441" s="2" t="n"/>
       <c r="E441" s="2" t="n"/>
       <c r="F441" s="2" t="n"/>
+      <c r="G441" s="2" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="2" t="n"/>
@@ -4128,6 +4591,7 @@
       <c r="D442" s="2" t="n"/>
       <c r="E442" s="2" t="n"/>
       <c r="F442" s="2" t="n"/>
+      <c r="G442" s="2" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="2" t="n"/>
@@ -4136,6 +4600,7 @@
       <c r="D443" s="2" t="n"/>
       <c r="E443" s="2" t="n"/>
       <c r="F443" s="2" t="n"/>
+      <c r="G443" s="2" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="2" t="n"/>
@@ -4144,6 +4609,7 @@
       <c r="D444" s="2" t="n"/>
       <c r="E444" s="2" t="n"/>
       <c r="F444" s="2" t="n"/>
+      <c r="G444" s="2" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="2" t="n"/>
@@ -4152,6 +4618,7 @@
       <c r="D445" s="2" t="n"/>
       <c r="E445" s="2" t="n"/>
       <c r="F445" s="2" t="n"/>
+      <c r="G445" s="2" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="2" t="n"/>
@@ -4160,6 +4627,7 @@
       <c r="D446" s="2" t="n"/>
       <c r="E446" s="2" t="n"/>
       <c r="F446" s="2" t="n"/>
+      <c r="G446" s="2" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="2" t="n"/>
@@ -4168,6 +4636,7 @@
       <c r="D447" s="2" t="n"/>
       <c r="E447" s="2" t="n"/>
       <c r="F447" s="2" t="n"/>
+      <c r="G447" s="2" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="2" t="n"/>
@@ -4176,6 +4645,7 @@
       <c r="D448" s="2" t="n"/>
       <c r="E448" s="2" t="n"/>
       <c r="F448" s="2" t="n"/>
+      <c r="G448" s="2" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="2" t="n"/>
@@ -4184,6 +4654,7 @@
       <c r="D449" s="2" t="n"/>
       <c r="E449" s="2" t="n"/>
       <c r="F449" s="2" t="n"/>
+      <c r="G449" s="2" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="2" t="n"/>
@@ -4192,6 +4663,7 @@
       <c r="D450" s="2" t="n"/>
       <c r="E450" s="2" t="n"/>
       <c r="F450" s="2" t="n"/>
+      <c r="G450" s="2" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="2" t="n"/>
@@ -4200,6 +4672,7 @@
       <c r="D451" s="2" t="n"/>
       <c r="E451" s="2" t="n"/>
       <c r="F451" s="2" t="n"/>
+      <c r="G451" s="2" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="2" t="n"/>
@@ -4208,6 +4681,7 @@
       <c r="D452" s="2" t="n"/>
       <c r="E452" s="2" t="n"/>
       <c r="F452" s="2" t="n"/>
+      <c r="G452" s="2" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="2" t="n"/>
@@ -4216,6 +4690,7 @@
       <c r="D453" s="2" t="n"/>
       <c r="E453" s="2" t="n"/>
       <c r="F453" s="2" t="n"/>
+      <c r="G453" s="2" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="2" t="n"/>
@@ -4224,6 +4699,7 @@
       <c r="D454" s="2" t="n"/>
       <c r="E454" s="2" t="n"/>
       <c r="F454" s="2" t="n"/>
+      <c r="G454" s="2" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="2" t="n"/>
@@ -4232,6 +4708,7 @@
       <c r="D455" s="2" t="n"/>
       <c r="E455" s="2" t="n"/>
       <c r="F455" s="2" t="n"/>
+      <c r="G455" s="2" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="n"/>
@@ -4240,6 +4717,7 @@
       <c r="D456" s="2" t="n"/>
       <c r="E456" s="2" t="n"/>
       <c r="F456" s="2" t="n"/>
+      <c r="G456" s="2" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="2" t="n"/>
@@ -4248,6 +4726,7 @@
       <c r="D457" s="2" t="n"/>
       <c r="E457" s="2" t="n"/>
       <c r="F457" s="2" t="n"/>
+      <c r="G457" s="2" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="2" t="n"/>
@@ -4256,6 +4735,7 @@
       <c r="D458" s="2" t="n"/>
       <c r="E458" s="2" t="n"/>
       <c r="F458" s="2" t="n"/>
+      <c r="G458" s="2" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="2" t="n"/>
@@ -4264,6 +4744,7 @@
       <c r="D459" s="2" t="n"/>
       <c r="E459" s="2" t="n"/>
       <c r="F459" s="2" t="n"/>
+      <c r="G459" s="2" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="2" t="n"/>
@@ -4272,6 +4753,7 @@
       <c r="D460" s="2" t="n"/>
       <c r="E460" s="2" t="n"/>
       <c r="F460" s="2" t="n"/>
+      <c r="G460" s="2" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="2" t="n"/>
@@ -4280,6 +4762,7 @@
       <c r="D461" s="2" t="n"/>
       <c r="E461" s="2" t="n"/>
       <c r="F461" s="2" t="n"/>
+      <c r="G461" s="2" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n"/>
@@ -4288,6 +4771,7 @@
       <c r="D462" s="2" t="n"/>
       <c r="E462" s="2" t="n"/>
       <c r="F462" s="2" t="n"/>
+      <c r="G462" s="2" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n"/>
@@ -4296,6 +4780,7 @@
       <c r="D463" s="2" t="n"/>
       <c r="E463" s="2" t="n"/>
       <c r="F463" s="2" t="n"/>
+      <c r="G463" s="2" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="2" t="n"/>
@@ -4304,6 +4789,7 @@
       <c r="D464" s="2" t="n"/>
       <c r="E464" s="2" t="n"/>
       <c r="F464" s="2" t="n"/>
+      <c r="G464" s="2" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="2" t="n"/>
@@ -4312,6 +4798,7 @@
       <c r="D465" s="2" t="n"/>
       <c r="E465" s="2" t="n"/>
       <c r="F465" s="2" t="n"/>
+      <c r="G465" s="2" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="2" t="n"/>
@@ -4320,6 +4807,7 @@
       <c r="D466" s="2" t="n"/>
       <c r="E466" s="2" t="n"/>
       <c r="F466" s="2" t="n"/>
+      <c r="G466" s="2" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="2" t="n"/>
@@ -4328,6 +4816,7 @@
       <c r="D467" s="2" t="n"/>
       <c r="E467" s="2" t="n"/>
       <c r="F467" s="2" t="n"/>
+      <c r="G467" s="2" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="2" t="n"/>
@@ -4336,6 +4825,7 @@
       <c r="D468" s="2" t="n"/>
       <c r="E468" s="2" t="n"/>
       <c r="F468" s="2" t="n"/>
+      <c r="G468" s="2" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="2" t="n"/>
@@ -4344,6 +4834,7 @@
       <c r="D469" s="2" t="n"/>
       <c r="E469" s="2" t="n"/>
       <c r="F469" s="2" t="n"/>
+      <c r="G469" s="2" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="2" t="n"/>
@@ -4352,6 +4843,7 @@
       <c r="D470" s="2" t="n"/>
       <c r="E470" s="2" t="n"/>
       <c r="F470" s="2" t="n"/>
+      <c r="G470" s="2" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="2" t="n"/>
@@ -4360,6 +4852,7 @@
       <c r="D471" s="2" t="n"/>
       <c r="E471" s="2" t="n"/>
       <c r="F471" s="2" t="n"/>
+      <c r="G471" s="2" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="2" t="n"/>
@@ -4368,6 +4861,7 @@
       <c r="D472" s="2" t="n"/>
       <c r="E472" s="2" t="n"/>
       <c r="F472" s="2" t="n"/>
+      <c r="G472" s="2" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="2" t="n"/>
@@ -4376,6 +4870,7 @@
       <c r="D473" s="2" t="n"/>
       <c r="E473" s="2" t="n"/>
       <c r="F473" s="2" t="n"/>
+      <c r="G473" s="2" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n"/>
@@ -4384,6 +4879,7 @@
       <c r="D474" s="2" t="n"/>
       <c r="E474" s="2" t="n"/>
       <c r="F474" s="2" t="n"/>
+      <c r="G474" s="2" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="2" t="n"/>
@@ -4392,6 +4888,7 @@
       <c r="D475" s="2" t="n"/>
       <c r="E475" s="2" t="n"/>
       <c r="F475" s="2" t="n"/>
+      <c r="G475" s="2" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n"/>
@@ -4400,6 +4897,7 @@
       <c r="D476" s="2" t="n"/>
       <c r="E476" s="2" t="n"/>
       <c r="F476" s="2" t="n"/>
+      <c r="G476" s="2" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="2" t="n"/>
@@ -4408,6 +4906,7 @@
       <c r="D477" s="2" t="n"/>
       <c r="E477" s="2" t="n"/>
       <c r="F477" s="2" t="n"/>
+      <c r="G477" s="2" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n"/>
@@ -4416,6 +4915,7 @@
       <c r="D478" s="2" t="n"/>
       <c r="E478" s="2" t="n"/>
       <c r="F478" s="2" t="n"/>
+      <c r="G478" s="2" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n"/>
@@ -4424,6 +4924,7 @@
       <c r="D479" s="2" t="n"/>
       <c r="E479" s="2" t="n"/>
       <c r="F479" s="2" t="n"/>
+      <c r="G479" s="2" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n"/>
@@ -4432,6 +4933,7 @@
       <c r="D480" s="2" t="n"/>
       <c r="E480" s="2" t="n"/>
       <c r="F480" s="2" t="n"/>
+      <c r="G480" s="2" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="2" t="n"/>
@@ -4440,6 +4942,7 @@
       <c r="D481" s="2" t="n"/>
       <c r="E481" s="2" t="n"/>
       <c r="F481" s="2" t="n"/>
+      <c r="G481" s="2" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="2" t="n"/>
@@ -4448,6 +4951,7 @@
       <c r="D482" s="2" t="n"/>
       <c r="E482" s="2" t="n"/>
       <c r="F482" s="2" t="n"/>
+      <c r="G482" s="2" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="2" t="n"/>
@@ -4456,6 +4960,7 @@
       <c r="D483" s="2" t="n"/>
       <c r="E483" s="2" t="n"/>
       <c r="F483" s="2" t="n"/>
+      <c r="G483" s="2" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="2" t="n"/>
@@ -4464,6 +4969,7 @@
       <c r="D484" s="2" t="n"/>
       <c r="E484" s="2" t="n"/>
       <c r="F484" s="2" t="n"/>
+      <c r="G484" s="2" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="2" t="n"/>
@@ -4472,6 +4978,7 @@
       <c r="D485" s="2" t="n"/>
       <c r="E485" s="2" t="n"/>
       <c r="F485" s="2" t="n"/>
+      <c r="G485" s="2" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="2" t="n"/>
@@ -4480,6 +4987,7 @@
       <c r="D486" s="2" t="n"/>
       <c r="E486" s="2" t="n"/>
       <c r="F486" s="2" t="n"/>
+      <c r="G486" s="2" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="2" t="n"/>
@@ -4488,6 +4996,7 @@
       <c r="D487" s="2" t="n"/>
       <c r="E487" s="2" t="n"/>
       <c r="F487" s="2" t="n"/>
+      <c r="G487" s="2" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="2" t="n"/>
@@ -4496,6 +5005,7 @@
       <c r="D488" s="2" t="n"/>
       <c r="E488" s="2" t="n"/>
       <c r="F488" s="2" t="n"/>
+      <c r="G488" s="2" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="2" t="n"/>
@@ -4504,6 +5014,7 @@
       <c r="D489" s="2" t="n"/>
       <c r="E489" s="2" t="n"/>
       <c r="F489" s="2" t="n"/>
+      <c r="G489" s="2" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n"/>
@@ -4512,6 +5023,7 @@
       <c r="D490" s="2" t="n"/>
       <c r="E490" s="2" t="n"/>
       <c r="F490" s="2" t="n"/>
+      <c r="G490" s="2" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="2" t="n"/>
@@ -4520,6 +5032,7 @@
       <c r="D491" s="2" t="n"/>
       <c r="E491" s="2" t="n"/>
       <c r="F491" s="2" t="n"/>
+      <c r="G491" s="2" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="2" t="n"/>
@@ -4528,6 +5041,7 @@
       <c r="D492" s="2" t="n"/>
       <c r="E492" s="2" t="n"/>
       <c r="F492" s="2" t="n"/>
+      <c r="G492" s="2" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="2" t="n"/>
@@ -4536,6 +5050,7 @@
       <c r="D493" s="2" t="n"/>
       <c r="E493" s="2" t="n"/>
       <c r="F493" s="2" t="n"/>
+      <c r="G493" s="2" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="2" t="n"/>
@@ -4544,6 +5059,7 @@
       <c r="D494" s="2" t="n"/>
       <c r="E494" s="2" t="n"/>
       <c r="F494" s="2" t="n"/>
+      <c r="G494" s="2" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="2" t="n"/>
@@ -4552,6 +5068,7 @@
       <c r="D495" s="2" t="n"/>
       <c r="E495" s="2" t="n"/>
       <c r="F495" s="2" t="n"/>
+      <c r="G495" s="2" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="n"/>
@@ -4560,6 +5077,7 @@
       <c r="D496" s="2" t="n"/>
       <c r="E496" s="2" t="n"/>
       <c r="F496" s="2" t="n"/>
+      <c r="G496" s="2" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="2" t="n"/>
@@ -4568,6 +5086,7 @@
       <c r="D497" s="2" t="n"/>
       <c r="E497" s="2" t="n"/>
       <c r="F497" s="2" t="n"/>
+      <c r="G497" s="2" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="2" t="n"/>
@@ -4576,6 +5095,7 @@
       <c r="D498" s="2" t="n"/>
       <c r="E498" s="2" t="n"/>
       <c r="F498" s="2" t="n"/>
+      <c r="G498" s="2" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="2" t="n"/>
@@ -4584,6 +5104,7 @@
       <c r="D499" s="2" t="n"/>
       <c r="E499" s="2" t="n"/>
       <c r="F499" s="2" t="n"/>
+      <c r="G499" s="2" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="2" t="n"/>
@@ -4592,6 +5113,7 @@
       <c r="D500" s="2" t="n"/>
       <c r="E500" s="2" t="n"/>
       <c r="F500" s="2" t="n"/>
+      <c r="G500" s="2" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="2" t="n"/>
@@ -4600,6 +5122,7 @@
       <c r="D501" s="2" t="n"/>
       <c r="E501" s="2" t="n"/>
       <c r="F501" s="2" t="n"/>
+      <c r="G501" s="2" t="n"/>
     </row>
     <row r="502">
       <c r="A502" s="2" t="n"/>
@@ -4608,6 +5131,7 @@
       <c r="D502" s="2" t="n"/>
       <c r="E502" s="2" t="n"/>
       <c r="F502" s="2" t="n"/>
+      <c r="G502" s="2" t="n"/>
     </row>
     <row r="503">
       <c r="A503" s="2" t="n"/>
@@ -4616,9 +5140,10 @@
       <c r="D503" s="2" t="n"/>
       <c r="E503" s="2" t="n"/>
       <c r="F503" s="2" t="n"/>
+      <c r="G503" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F503"/>
+  <autoFilter ref="A1:G503"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -4630,7 +5155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4709,7 +5234,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>telefono</t>
+          <t>rfc</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -4719,31 +5244,31 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Telefono del promotor.</t>
+          <t>RFC obligatorio para identificar historico aunque se repita el nombre.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>supervisor</t>
+          <t>telefono</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Referencia opcional. Puede ser nombre, email o numero de empleado del supervisor.</t>
+          <t>Telefono del promotor.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>contrasena</t>
+          <t>supervisor</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -4753,12 +5278,29 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
+          <t>Referencia opcional. Puede ser nombre, email o numero de empleado del supervisor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>contrasena</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>Si se deja vacia, se usa la contrasena default capturada en el panel.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C7"/>
+  <autoFilter ref="A1:C8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>